<commit_message>
Modificacion de archivos segun correciones marcadas
</commit_message>
<xml_diff>
--- a/01 Documentación/Scrum/Sprint I/EcoWaste_Product_Backlog Sprint I.xlsx
+++ b/01 Documentación/Scrum/Sprint I/EcoWaste_Product_Backlog Sprint I.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dbc_1\Documents\Desarrollo de software\presentación 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Documents\EcoWaste\ProyectoEcoWaste\01 Documentación\Scrum\Sprint I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393D1C7B-9773-42E2-94E7-F0631F3D7B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96874780-CC27-45F5-9DDC-9A18258932AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FDDBCD3E-BA3F-4940-BC94-5DDA34DAB6C1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FDDBCD3E-BA3F-4940-BC94-5DDA34DAB6C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -369,7 +369,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -387,24 +387,14 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF990000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF7F6000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF38761D"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -414,13 +404,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF990000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -439,7 +422,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -466,6 +449,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8F8F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -520,7 +509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -534,53 +523,59 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -917,39 +912,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7390B81B-38B2-473A-92B1-80DE68A05723}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" style="20" customWidth="1"/>
+    <col min="1" max="1" width="1.88671875" style="15" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="72.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-    <col min="9" max="9" width="53.140625" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="17"/>
+    <col min="3" max="3" width="72.88671875" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" customWidth="1"/>
+    <col min="5" max="8" width="11.5546875"/>
+    <col min="9" max="9" width="53.109375" customWidth="1"/>
+    <col min="10" max="16384" width="11.44140625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="18" t="s">
+    <row r="1" spans="2:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-    </row>
-    <row r="2" spans="2:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-    </row>
-    <row r="3" spans="2:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+    </row>
+    <row r="2" spans="2:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+    </row>
+    <row r="3" spans="2:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -975,256 +971,268 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="9" t="s">
+    <row r="4" spans="2:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="19">
         <v>58</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="17">
         <v>1</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="9" t="s">
+      <c r="I4" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="19">
         <v>19</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="17">
         <v>2</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="9" t="s">
+      <c r="I5" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="19">
         <v>38</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="17">
         <v>3</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
+      <c r="I6" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="19">
         <v>19</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="17">
         <v>4</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="9" t="s">
+      <c r="I7" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="21">
         <v>29</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="22">
         <v>5</v>
       </c>
-      <c r="I8" s="6"/>
-    </row>
-    <row r="9" spans="2:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="9" t="s">
+      <c r="I8" s="20"/>
+    </row>
+    <row r="9" spans="2:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="21">
         <v>29</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="22">
         <v>6</v>
       </c>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="9" t="s">
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15"/>
-    </row>
-    <row r="11" spans="2:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="9" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="4">
+        <v>7</v>
+      </c>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="2:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="12" t="s">
         <v>90</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12" spans="2:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="9" t="s">
+      <c r="E11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="4">
+        <v>8</v>
+      </c>
+      <c r="I11" s="12"/>
+    </row>
+    <row r="12" spans="2:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="12" t="s">
         <v>92</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="16"/>
-    </row>
-    <row r="13" spans="2:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="9" t="s">
+      <c r="E12" s="8"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="4">
+        <v>9</v>
+      </c>
+      <c r="I12" s="12"/>
+    </row>
+    <row r="13" spans="2:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="12" t="s">
         <v>94</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="4"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="4">
+        <v>10</v>
+      </c>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="9" t="s">
+    <row r="14" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="12" t="s">
         <v>96</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="4"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="4">
+        <v>11</v>
+      </c>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="2:9" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="9" t="s">
+    <row r="15" spans="2:9" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="12" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="4"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="4">
+        <v>12</v>
+      </c>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="9" t="s">
+    <row r="16" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1236,13 +1244,15 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="4"/>
+      <c r="H16" s="4">
+        <v>13</v>
+      </c>
       <c r="I16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
+    <row r="17" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1254,31 +1264,35 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="5"/>
+      <c r="H17" s="4">
+        <v>14</v>
+      </c>
       <c r="I17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
+    <row r="18" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="3"/>
-      <c r="F18" s="7"/>
+      <c r="F18" s="6"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B19" s="9" t="s">
+      <c r="H18" s="4">
+        <v>15</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="7" t="s">
         <v>50</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1290,13 +1304,15 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="8"/>
+      <c r="H19" s="4">
+        <v>16</v>
+      </c>
       <c r="I19" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B20" s="9" t="s">
+    <row r="20" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="7" t="s">
         <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1308,31 +1324,35 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="H20" s="4"/>
+      <c r="H20" s="4">
+        <v>17</v>
+      </c>
       <c r="I20" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B21" s="9" t="s">
+    <row r="21" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B21" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="3"/>
-      <c r="F21" s="7"/>
+      <c r="F21" s="6"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B22" s="9" t="s">
+      <c r="H21" s="4">
+        <v>18</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B22" s="7" t="s">
         <v>105</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -1343,14 +1363,16 @@
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="8"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="4">
+        <v>19</v>
+      </c>
       <c r="I22" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B23" s="9" t="s">
+    <row r="23" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="7" t="s">
         <v>106</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -1361,14 +1383,16 @@
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="8"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="4">
+        <v>20</v>
+      </c>
       <c r="I23" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B24" s="9" t="s">
+    <row r="24" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B24" s="7" t="s">
         <v>56</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -1379,14 +1403,16 @@
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="8"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="4">
+        <v>21</v>
+      </c>
       <c r="I24" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
+    <row r="25" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B25" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -1397,50 +1423,56 @@
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="8"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="4">
+        <v>22</v>
+      </c>
       <c r="I25" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B26" s="9" t="s">
+    <row r="26" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B26" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>55</v>
       </c>
       <c r="E26" s="3"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B27" s="9" t="s">
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="4">
+        <v>23</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B27" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E27" s="3"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B28" s="9" t="s">
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="4">
+        <v>24</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B28" s="7" t="s">
         <v>68</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -1451,32 +1483,36 @@
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="5"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="4">
+        <v>25</v>
+      </c>
       <c r="I28" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B29" s="9" t="s">
+    <row r="29" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B29" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>64</v>
       </c>
       <c r="E29" s="3"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="4">
+        <v>26</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="7" t="s">
         <v>74</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1487,32 +1523,36 @@
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="5"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="4">
+        <v>27</v>
+      </c>
       <c r="I30" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
+    <row r="31" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B31" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="6" t="s">
         <v>70</v>
       </c>
       <c r="E31" s="3"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B32" s="9" t="s">
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="4">
+        <v>28</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B32" s="7" t="s">
         <v>80</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -1523,32 +1563,36 @@
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="5"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="4">
+        <v>29</v>
+      </c>
       <c r="I32" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B33" s="9" t="s">
+    <row r="33" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B33" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="6" t="s">
         <v>76</v>
       </c>
       <c r="E33" s="3"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="2:9" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B34" s="9" t="s">
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="4">
+        <v>30</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B34" s="7" t="s">
         <v>86</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -1559,14 +1603,16 @@
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="8"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="4">
+        <v>31</v>
+      </c>
       <c r="I34" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="2:9" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B35" s="9" t="s">
+    <row r="35" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B35" s="7" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -1578,7 +1624,9 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
-      <c r="H35" s="5"/>
+      <c r="H35" s="4">
+        <v>32</v>
+      </c>
       <c r="I35" s="2" t="s">
         <v>11</v>
       </c>
@@ -1589,7 +1637,7 @@
     <mergeCell ref="A1:A1048576"/>
     <mergeCell ref="J1:XFD1048576"/>
   </mergeCells>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>